<commit_message>
Fill in Company for per-company catalog rows and reject duplicates
Basic Pay, Guaranteed Bonus and MTS Recovery each had one row per
company but a blank Company column, so the catalog upload gave them the
same id and kept only the last row - 359 workbook rows became 354 line
items. Company is now set from the cost center (81 OCC, 80 OCLP,
90 OLC), and the upload rejects rows sharing category + name + company,
naming the sheet rows, instead of silently overwriting them.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Budgeting System_Expense Line Items.xlsx
+++ b/Budgeting System_Expense Line Items.xlsx
@@ -3889,6 +3889,11 @@
       <c r="F38" s="5" t="s">
         <v>502</v>
       </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>OCC</t>
+        </is>
+      </c>
       <c r="I38" t="s">
         <v>443</v>
       </c>
@@ -3930,6 +3935,11 @@
       <c r="F39" s="5" t="s">
         <v>502</v>
       </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>OCLP</t>
+        </is>
+      </c>
       <c r="I39" t="s">
         <v>443</v>
       </c>
@@ -10839,6 +10849,11 @@
       <c r="F195" s="5" t="s">
         <v>341</v>
       </c>
+      <c r="G195" s="5" t="inlineStr">
+        <is>
+          <t>OCC</t>
+        </is>
+      </c>
       <c r="I195" t="s">
         <v>84</v>
       </c>
@@ -10880,6 +10895,11 @@
       <c r="F196" s="5" t="s">
         <v>341</v>
       </c>
+      <c r="G196" s="5" t="inlineStr">
+        <is>
+          <t>OCLP</t>
+        </is>
+      </c>
       <c r="I196" t="s">
         <v>84</v>
       </c>
@@ -10921,6 +10941,11 @@
       <c r="F197" s="5" t="s">
         <v>341</v>
       </c>
+      <c r="G197" s="5" t="inlineStr">
+        <is>
+          <t>OLC</t>
+        </is>
+      </c>
       <c r="I197" t="s">
         <v>84</v>
       </c>
@@ -11367,6 +11392,11 @@
       <c r="F207" s="5" t="s">
         <v>342</v>
       </c>
+      <c r="G207" s="5" t="inlineStr">
+        <is>
+          <t>OCC</t>
+        </is>
+      </c>
       <c r="I207" t="s">
         <v>84</v>
       </c>
@@ -11408,6 +11438,11 @@
       <c r="F208" s="5" t="s">
         <v>342</v>
       </c>
+      <c r="G208" s="5" t="inlineStr">
+        <is>
+          <t>OCLP</t>
+        </is>
+      </c>
       <c r="I208" t="s">
         <v>84</v>
       </c>
@@ -11448,6 +11483,11 @@
       </c>
       <c r="F209" s="5" t="s">
         <v>342</v>
+      </c>
+      <c r="G209" s="5" t="inlineStr">
+        <is>
+          <t>OLC</t>
+        </is>
       </c>
       <c r="I209" t="s">
         <v>84</v>

</xml_diff>

<commit_message>
Make 8 OMD Operations line items visible to every department
Clears the "visible only to OMD Operations" restriction (column R) for
Kitchen Equipment, Office Equipment, Others, Toner/Ink, Building,
Furniture, Fixture & Equipment, Supplies and Vehicle in the Expense
Line Items workbook, and syncs the seed copy.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Budgeting System_Expense Line Items.xlsx
+++ b/Budgeting System_Expense Line Items.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jumalonpvp\Downloads\Budgeting System\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E22C5CD5-4330-4943-873D-82AB26DC2A8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D336090E-2934-4E30-BA17-06665BAB9329}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7D30BD04-AED0-48C4-A0F0-DC51EF4C24C2}"/>
   </bookViews>
@@ -3889,10 +3889,8 @@
       <c r="F38" s="5" t="s">
         <v>502</v>
       </c>
-      <c r="G38" s="5" t="inlineStr">
-        <is>
-          <t>OCC</t>
-        </is>
+      <c r="G38" s="5" t="s">
+        <v>219</v>
       </c>
       <c r="I38" t="s">
         <v>443</v>
@@ -3935,10 +3933,8 @@
       <c r="F39" s="5" t="s">
         <v>502</v>
       </c>
-      <c r="G39" s="5" t="inlineStr">
-        <is>
-          <t>OCLP</t>
-        </is>
+      <c r="G39" s="5" t="s">
+        <v>220</v>
       </c>
       <c r="I39" t="s">
         <v>443</v>
@@ -10849,10 +10845,8 @@
       <c r="F195" s="5" t="s">
         <v>341</v>
       </c>
-      <c r="G195" s="5" t="inlineStr">
-        <is>
-          <t>OCC</t>
-        </is>
+      <c r="G195" s="5" t="s">
+        <v>219</v>
       </c>
       <c r="I195" t="s">
         <v>84</v>
@@ -10895,10 +10889,8 @@
       <c r="F196" s="5" t="s">
         <v>341</v>
       </c>
-      <c r="G196" s="5" t="inlineStr">
-        <is>
-          <t>OCLP</t>
-        </is>
+      <c r="G196" s="5" t="s">
+        <v>220</v>
       </c>
       <c r="I196" t="s">
         <v>84</v>
@@ -10941,10 +10933,8 @@
       <c r="F197" s="5" t="s">
         <v>341</v>
       </c>
-      <c r="G197" s="5" t="inlineStr">
-        <is>
-          <t>OLC</t>
-        </is>
+      <c r="G197" s="5" t="s">
+        <v>221</v>
       </c>
       <c r="I197" t="s">
         <v>84</v>
@@ -11392,10 +11382,8 @@
       <c r="F207" s="5" t="s">
         <v>342</v>
       </c>
-      <c r="G207" s="5" t="inlineStr">
-        <is>
-          <t>OCC</t>
-        </is>
+      <c r="G207" s="5" t="s">
+        <v>219</v>
       </c>
       <c r="I207" t="s">
         <v>84</v>
@@ -11438,10 +11426,8 @@
       <c r="F208" s="5" t="s">
         <v>342</v>
       </c>
-      <c r="G208" s="5" t="inlineStr">
-        <is>
-          <t>OCLP</t>
-        </is>
+      <c r="G208" s="5" t="s">
+        <v>220</v>
       </c>
       <c r="I208" t="s">
         <v>84</v>
@@ -11484,10 +11470,8 @@
       <c r="F209" s="5" t="s">
         <v>342</v>
       </c>
-      <c r="G209" s="5" t="inlineStr">
-        <is>
-          <t>OLC</t>
-        </is>
+      <c r="G209" s="5" t="s">
+        <v>221</v>
       </c>
       <c r="I209" t="s">
         <v>84</v>
@@ -16529,9 +16513,6 @@
       <c r="M329">
         <v>52111102</v>
       </c>
-      <c r="R329" t="s">
-        <v>300</v>
-      </c>
     </row>
     <row r="330" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A330" t="str">
@@ -16570,9 +16551,6 @@
       <c r="M330">
         <v>52111102</v>
       </c>
-      <c r="R330" t="s">
-        <v>300</v>
-      </c>
     </row>
     <row r="331" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A331" t="str">
@@ -16614,9 +16592,6 @@
       <c r="N331" t="s">
         <v>249</v>
       </c>
-      <c r="R331" t="s">
-        <v>300</v>
-      </c>
     </row>
     <row r="332" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A332" t="str">
@@ -16655,9 +16630,6 @@
       <c r="M332">
         <v>52111101</v>
       </c>
-      <c r="R332" t="s">
-        <v>300</v>
-      </c>
     </row>
     <row r="333" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A333" t="str">
@@ -16696,9 +16668,6 @@
       <c r="M333">
         <v>52061103</v>
       </c>
-      <c r="R333" t="s">
-        <v>300</v>
-      </c>
     </row>
     <row r="334" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A334" t="str">
@@ -16737,9 +16706,6 @@
       <c r="M334">
         <v>52061101</v>
       </c>
-      <c r="R334" t="s">
-        <v>300</v>
-      </c>
     </row>
     <row r="335" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A335" t="str">
@@ -16778,9 +16744,6 @@
       <c r="M335">
         <v>52061103</v>
       </c>
-      <c r="R335" t="s">
-        <v>300</v>
-      </c>
     </row>
     <row r="336" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A336" t="str">
@@ -16818,9 +16781,6 @@
       </c>
       <c r="M336">
         <v>52061105</v>
-      </c>
-      <c r="R336" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="337" spans="1:18" x14ac:dyDescent="0.35">

</xml_diff>